<commit_message>
Jubecer: guards list filters/pagination, dashboard KPIs, requirements upload/download, schema updates
</commit_message>
<xml_diff>
--- a/remarks.xlsx
+++ b/remarks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Acer\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\ERMS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{386E65A7-F9E5-4FC5-AE2F-0E0FC4AE25BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4946FF34-9184-4F5D-90AA-43091B7D3F81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1737,19 +1737,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C146"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="9.109375" style="1"/>
-    <col min="3" max="3" width="127.44140625" style="1" customWidth="1"/>
-    <col min="4" max="16384" width="9.109375" style="1"/>
+    <col min="1" max="2" width="9.140625" style="1"/>
+    <col min="3" max="3" width="127.42578125" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2">
         <v>1</v>
@@ -1758,7 +1758,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="2">
         <v>2</v>
@@ -1767,7 +1767,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2">
         <v>3</v>
@@ -1776,7 +1776,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="2">
         <v>4</v>
@@ -1785,7 +1785,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2">
         <v>5</v>
@@ -1794,12 +1794,12 @@
         <v>433</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="3"/>
     </row>
-    <row r="8" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2">
         <v>8</v>
@@ -1808,12 +1808,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
     </row>
-    <row r="10" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2">
         <v>11</v>
@@ -1822,7 +1822,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2">
         <v>12</v>
@@ -1831,7 +1831,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2">
         <v>13</v>
@@ -1840,7 +1840,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2">
         <v>14</v>
@@ -1849,7 +1849,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2">
         <v>15</v>
@@ -1858,7 +1858,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2">
         <v>16</v>
@@ -1867,7 +1867,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2">
         <v>17</v>
@@ -1876,7 +1876,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2">
         <v>18</v>
@@ -1885,7 +1885,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2">
         <v>19</v>
@@ -1894,12 +1894,12 @@
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="3"/>
     </row>
-    <row r="20" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2">
         <v>138</v>
@@ -1908,7 +1908,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" s="2">
         <v>139</v>
@@ -1917,7 +1917,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
       <c r="B22" s="2">
         <v>140</v>
@@ -1926,7 +1926,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
       <c r="B23" s="2">
         <v>141</v>
@@ -1935,7 +1935,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="2">
         <v>172</v>
@@ -1944,12 +1944,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="3"/>
     </row>
-    <row r="26" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
       <c r="B26" s="2">
         <v>174</v>
@@ -1958,7 +1958,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
       <c r="B27" s="2">
         <v>175</v>
@@ -1967,7 +1967,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
       <c r="B28" s="2">
         <v>176</v>
@@ -1976,12 +1976,12 @@
         <v>36</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="3"/>
     </row>
-    <row r="30" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
       <c r="B30" s="2">
         <v>178</v>
@@ -1990,7 +1990,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
       <c r="B31" s="2">
         <v>179</v>
@@ -1999,7 +1999,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="2">
         <v>180</v>
@@ -2008,7 +2008,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
       <c r="B33" s="2">
         <v>181</v>
@@ -2017,7 +2017,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="2">
         <v>182</v>
@@ -2026,7 +2026,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="2">
         <v>183</v>
@@ -2035,7 +2035,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="2">
         <v>184</v>
@@ -2044,12 +2044,12 @@
         <v>56</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="3"/>
     </row>
-    <row r="38" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
       <c r="B38" s="2">
         <v>186</v>
@@ -2058,7 +2058,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="2"/>
       <c r="B39" s="2">
         <v>187</v>
@@ -2067,7 +2067,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
       <c r="B40" s="2">
         <v>188</v>
@@ -2076,12 +2076,12 @@
         <v>176</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
     </row>
-    <row r="42" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
       <c r="B42" s="2">
         <v>191</v>
@@ -2090,7 +2090,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="2"/>
       <c r="B43" s="2">
         <v>192</v>
@@ -2099,7 +2099,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="2"/>
       <c r="B44" s="2">
         <v>193</v>
@@ -2108,7 +2108,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="2"/>
       <c r="B45" s="2">
         <v>194</v>
@@ -2117,19 +2117,19 @@
         <v>195</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="3" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="3"/>
     </row>
-    <row r="48" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" s="2"/>
       <c r="B48" s="2">
         <v>197</v>
@@ -2138,7 +2138,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" s="2"/>
       <c r="B49" s="2">
         <v>198</v>
@@ -2147,24 +2147,24 @@
         <v>186</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="3" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="3"/>
     </row>
-    <row r="52" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="3"/>
     </row>
-    <row r="53" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A53" s="2"/>
       <c r="B53" s="2">
         <v>200</v>
@@ -2173,7 +2173,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A54" s="2"/>
       <c r="B54" s="2">
         <v>201</v>
@@ -2182,12 +2182,12 @@
         <v>152</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
     </row>
-    <row r="56" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A56" s="2"/>
       <c r="B56" s="2">
         <v>203</v>
@@ -2196,12 +2196,12 @@
         <v>29</v>
       </c>
     </row>
-    <row r="57" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
     </row>
-    <row r="58" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A58" s="2"/>
       <c r="B58" s="2">
         <v>205</v>
@@ -2210,7 +2210,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A59" s="2"/>
       <c r="B59" s="2">
         <v>208</v>
@@ -2219,7 +2219,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A60" s="2"/>
       <c r="B60" s="2">
         <v>206</v>
@@ -2228,7 +2228,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A61" s="2"/>
       <c r="B61" s="2">
         <v>209</v>
@@ -2237,21 +2237,21 @@
         <v>134</v>
       </c>
     </row>
-    <row r="62" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="3" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="63" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="3" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="64" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A64" s="2"/>
       <c r="B64" s="2">
         <v>207</v>
@@ -2260,17 +2260,17 @@
         <v>71</v>
       </c>
     </row>
-    <row r="65" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="3"/>
     </row>
-    <row r="66" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A66" s="2"/>
       <c r="B66" s="2"/>
       <c r="C66" s="3"/>
     </row>
-    <row r="67" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A67" s="2"/>
       <c r="B67" s="2">
         <v>212</v>
@@ -2279,7 +2279,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="68" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A68" s="2"/>
       <c r="B68" s="2">
         <v>213</v>
@@ -2288,7 +2288,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="69" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A69" s="2"/>
       <c r="B69" s="2">
         <v>214</v>
@@ -2297,12 +2297,12 @@
         <v>63</v>
       </c>
     </row>
-    <row r="70" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A70" s="2"/>
       <c r="B70" s="2"/>
       <c r="C70" s="3"/>
     </row>
-    <row r="71" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A71" s="2"/>
       <c r="B71" s="2">
         <v>216</v>
@@ -2311,7 +2311,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="72" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A72" s="2"/>
       <c r="B72" s="2">
         <v>217</v>
@@ -2320,12 +2320,12 @@
         <v>37</v>
       </c>
     </row>
-    <row r="73" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
     </row>
-    <row r="74" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A74" s="2"/>
       <c r="B74" s="2">
         <v>219</v>
@@ -2334,12 +2334,12 @@
         <v>38</v>
       </c>
     </row>
-    <row r="75" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
     </row>
-    <row r="76" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A76" s="2"/>
       <c r="B76" s="2">
         <v>221</v>
@@ -2348,7 +2348,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="77" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A77" s="2"/>
       <c r="B77" s="2">
         <v>222</v>
@@ -2357,12 +2357,12 @@
         <v>197</v>
       </c>
     </row>
-    <row r="78" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
     </row>
-    <row r="79" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A79" s="2"/>
       <c r="B79" s="2">
         <v>226</v>
@@ -2371,7 +2371,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="80" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A80" s="2"/>
       <c r="B80" s="2">
         <v>227</v>
@@ -2380,19 +2380,19 @@
         <v>82</v>
       </c>
     </row>
-    <row r="81" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
       <c r="C81" s="3" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A82" s="2"/>
       <c r="B82" s="2"/>
       <c r="C82" s="3"/>
     </row>
-    <row r="83" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A83" s="2"/>
       <c r="B83" s="2">
         <v>230</v>
@@ -2401,12 +2401,12 @@
         <v>51</v>
       </c>
     </row>
-    <row r="84" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A84" s="2"/>
       <c r="B84" s="2"/>
       <c r="C84" s="2"/>
     </row>
-    <row r="85" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A85" s="2"/>
       <c r="B85" s="2">
         <v>232</v>
@@ -2415,7 +2415,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="86" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A86" s="2"/>
       <c r="B86" s="2">
         <v>233</v>
@@ -2424,7 +2424,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="87" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A87" s="2"/>
       <c r="B87" s="2">
         <v>234</v>
@@ -2433,7 +2433,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="88" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A88" s="2"/>
       <c r="B88" s="2">
         <v>235</v>
@@ -2442,7 +2442,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="89" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A89" s="2"/>
       <c r="B89" s="2">
         <v>236</v>
@@ -2451,19 +2451,19 @@
         <v>181</v>
       </c>
     </row>
-    <row r="90" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A90" s="2"/>
       <c r="B90" s="2"/>
       <c r="C90" s="3" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="91" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="3"/>
     </row>
-    <row r="92" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A92" s="2"/>
       <c r="B92" s="2">
         <v>239</v>
@@ -2472,12 +2472,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="93" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="3"/>
     </row>
-    <row r="94" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A94" s="2"/>
       <c r="B94" s="2">
         <v>243</v>
@@ -2486,12 +2486,12 @@
         <v>70</v>
       </c>
     </row>
-    <row r="95" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
     </row>
-    <row r="96" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A96" s="2"/>
       <c r="B96" s="2">
         <v>245</v>
@@ -2500,7 +2500,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="97" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A97" s="2"/>
       <c r="B97" s="2">
         <v>246</v>
@@ -2509,12 +2509,12 @@
         <v>175</v>
       </c>
     </row>
-    <row r="98" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="3"/>
     </row>
-    <row r="99" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A99" s="2"/>
       <c r="B99" s="2">
         <v>249</v>
@@ -2523,7 +2523,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="100" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A100" s="2"/>
       <c r="B100" s="2">
         <v>250</v>
@@ -2532,7 +2532,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="101" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A101" s="2"/>
       <c r="B101" s="2">
         <v>251</v>
@@ -2541,12 +2541,12 @@
         <v>81</v>
       </c>
     </row>
-    <row r="102" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A102" s="2"/>
       <c r="B102" s="2"/>
       <c r="C102" s="3"/>
     </row>
-    <row r="103" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A103" s="2"/>
       <c r="B103" s="2">
         <v>254</v>
@@ -2555,7 +2555,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="104" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A104" s="2"/>
       <c r="B104" s="2">
         <v>256</v>
@@ -2564,12 +2564,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="105" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A105" s="2"/>
       <c r="B105" s="2"/>
       <c r="C105" s="3"/>
     </row>
-    <row r="106" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A106" s="2"/>
       <c r="B106" s="2">
         <v>258</v>
@@ -2578,19 +2578,19 @@
         <v>113</v>
       </c>
     </row>
-    <row r="107" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A107" s="2"/>
       <c r="B107" s="2"/>
       <c r="C107" s="3" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="108" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A108" s="2"/>
       <c r="B108" s="2"/>
       <c r="C108" s="3"/>
     </row>
-    <row r="109" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A109" s="2"/>
       <c r="B109" s="2">
         <v>260</v>
@@ -2599,7 +2599,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="110" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A110" s="2"/>
       <c r="B110" s="2">
         <v>261</v>
@@ -2608,13 +2608,13 @@
         <v>165</v>
       </c>
     </row>
-    <row r="111" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A111" s="2"/>
       <c r="B111" s="2">
         <v>263</v>
       </c>
     </row>
-    <row r="112" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A112" s="2"/>
       <c r="B112" s="2">
         <v>265</v>
@@ -2623,7 +2623,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="113" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A113" s="2"/>
       <c r="B113" s="2">
         <v>266</v>
@@ -2632,12 +2632,12 @@
         <v>196</v>
       </c>
     </row>
-    <row r="114" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A114" s="2"/>
       <c r="B114" s="2"/>
       <c r="C114" s="2"/>
     </row>
-    <row r="115" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A115" s="2"/>
       <c r="B115" s="2">
         <v>267</v>
@@ -2646,7 +2646,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="116" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A116" s="2"/>
       <c r="B116" s="2">
         <v>268</v>
@@ -2655,12 +2655,12 @@
         <v>35</v>
       </c>
     </row>
-    <row r="117" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A117" s="2"/>
       <c r="B117" s="2"/>
       <c r="C117" s="3"/>
     </row>
-    <row r="118" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B118" s="2">
         <v>270</v>
       </c>
@@ -2668,11 +2668,11 @@
         <v>7</v>
       </c>
     </row>
-    <row r="119" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B119" s="2"/>
       <c r="C119" s="2"/>
     </row>
-    <row r="120" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B120" s="2">
         <v>272</v>
       </c>
@@ -2680,7 +2680,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="121" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B121" s="2">
         <v>273</v>
       </c>
@@ -2688,11 +2688,11 @@
         <v>190</v>
       </c>
     </row>
-    <row r="122" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B122" s="2"/>
       <c r="C122" s="2"/>
     </row>
-    <row r="123" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B123" s="2">
         <v>276</v>
       </c>
@@ -2700,50 +2700,50 @@
         <v>192</v>
       </c>
     </row>
-    <row r="124" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C124" s="2" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="127" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C127" s="3" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="128" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C128" s="3"/>
     </row>
-    <row r="129" spans="3:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="129" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C129" s="3" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="131" spans="3:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="131" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C131" s="3" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="132" spans="3:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="132" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C132" s="3" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="134" spans="3:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="134" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C134" s="3" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="136" spans="3:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="136" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C136" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="137" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="137" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C137" s="1" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="146" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="146" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C146" s="6" t="s">
         <v>435</v>
       </c>
@@ -2760,12 +2760,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B3:C58"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="9.109375" style="1"/>
+    <col min="1" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="2">
         <v>1</v>
       </c>
@@ -2773,7 +2773,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="4" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B4" s="2">
         <v>3</v>
       </c>
@@ -2781,7 +2781,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="5" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="2">
         <v>4</v>
       </c>
@@ -2789,7 +2789,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="6" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B6" s="2">
         <v>6</v>
       </c>
@@ -2797,7 +2797,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="7" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B7" s="2">
         <v>8</v>
       </c>
@@ -2805,7 +2805,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="8" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B8" s="2">
         <v>9</v>
       </c>
@@ -2813,7 +2813,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="2">
         <v>10</v>
       </c>
@@ -2821,7 +2821,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B10" s="2">
         <v>11</v>
       </c>
@@ -2829,7 +2829,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="11" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B11" s="2">
         <v>12</v>
       </c>
@@ -2837,7 +2837,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="12" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B12" s="2">
         <v>13</v>
       </c>
@@ -2845,7 +2845,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B13" s="2">
         <v>15</v>
       </c>
@@ -2853,7 +2853,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="14" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B14" s="2">
         <v>16</v>
       </c>
@@ -2861,7 +2861,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="15" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B15" s="2">
         <v>17</v>
       </c>
@@ -2869,7 +2869,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="16" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B16" s="2">
         <v>18</v>
       </c>
@@ -2877,7 +2877,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B17" s="2">
         <v>19</v>
       </c>
@@ -2885,7 +2885,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="18" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B18" s="2">
         <v>20</v>
       </c>
@@ -2893,7 +2893,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="19" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B19" s="2">
         <v>21</v>
       </c>
@@ -2901,7 +2901,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="20" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B20" s="2">
         <v>22</v>
       </c>
@@ -2909,7 +2909,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="21" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B21" s="2">
         <v>24</v>
       </c>
@@ -2917,7 +2917,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="22" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B22" s="2">
         <v>27</v>
       </c>
@@ -2925,7 +2925,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="23" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B23" s="2">
         <v>28</v>
       </c>
@@ -2933,7 +2933,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="24" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B24" s="2">
         <v>29</v>
       </c>
@@ -2941,7 +2941,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="25" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B25" s="2">
         <v>30</v>
       </c>
@@ -2949,7 +2949,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B26" s="2">
         <v>31</v>
       </c>
@@ -2957,7 +2957,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B27" s="2">
         <v>32</v>
       </c>
@@ -2965,7 +2965,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="28" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B28" s="2">
         <v>33</v>
       </c>
@@ -2973,7 +2973,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="29" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B29" s="2">
         <v>34</v>
       </c>
@@ -2981,7 +2981,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="30" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B30" s="2">
         <v>35</v>
       </c>
@@ -2989,7 +2989,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="31" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B31" s="2">
         <v>36</v>
       </c>
@@ -2997,7 +2997,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="32" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B32" s="2">
         <v>37</v>
       </c>
@@ -3005,7 +3005,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="33" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B33" s="2">
         <v>38</v>
       </c>
@@ -3013,7 +3013,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="34" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B34" s="2">
         <v>39</v>
       </c>
@@ -3021,7 +3021,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="35" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B35" s="2">
         <v>42</v>
       </c>
@@ -3029,7 +3029,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="36" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B36" s="2">
         <v>43</v>
       </c>
@@ -3037,7 +3037,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="37" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B37" s="2">
         <v>45</v>
       </c>
@@ -3045,7 +3045,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="38" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B38" s="2">
         <v>46</v>
       </c>
@@ -3053,7 +3053,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="39" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B39" s="2">
         <v>47</v>
       </c>
@@ -3061,7 +3061,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="40" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B40" s="2">
         <v>48</v>
       </c>
@@ -3069,7 +3069,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="41" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B41" s="2">
         <v>49</v>
       </c>
@@ -3077,7 +3077,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="42" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B42" s="2">
         <v>50</v>
       </c>
@@ -3085,82 +3085,82 @@
         <v>199</v>
       </c>
     </row>
-    <row r="43" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C43" s="3" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="44" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C44" s="2" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="45" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C45" s="3" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="46" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C46" s="3" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="47" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C47" s="3" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="48" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C48" s="3" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="49" spans="3:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C49" s="2" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="50" spans="3:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C50" s="2" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="51" spans="3:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C51" s="3" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="52" spans="3:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="52" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C52" s="3" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="53" spans="3:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="53" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C53" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="54" spans="3:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="54" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C54" s="2" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="55" spans="3:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="55" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C55" s="3" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="56" spans="3:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="56" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C56" s="2" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="57" spans="3:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="57" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C57" s="4" t="s">
         <v>437</v>
       </c>
     </row>
-    <row r="58" spans="3:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="58" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C58" s="3" t="s">
         <v>433</v>
       </c>
@@ -3170,19 +3170,19 @@
     <sortCondition ref="C8"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B4:C78"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="9.109375" style="1"/>
+    <col min="1" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B4" s="2">
         <v>1</v>
       </c>
@@ -3190,7 +3190,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="5" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="2">
         <v>3</v>
       </c>
@@ -3198,7 +3198,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="6" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B6" s="2">
         <v>4</v>
       </c>
@@ -3206,7 +3206,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="7" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B7" s="2">
         <v>5</v>
       </c>
@@ -3214,7 +3214,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="8" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B8" s="2">
         <v>6</v>
       </c>
@@ -3222,7 +3222,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="2">
         <v>7</v>
       </c>
@@ -3230,7 +3230,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="10" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B10" s="2">
         <v>8</v>
       </c>
@@ -3238,7 +3238,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="11" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B11" s="2">
         <v>9</v>
       </c>
@@ -3246,7 +3246,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B12" s="2">
         <v>10</v>
       </c>
@@ -3254,7 +3254,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="13" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B13" s="2">
         <v>11</v>
       </c>
@@ -3262,7 +3262,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="14" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B14" s="2">
         <v>12</v>
       </c>
@@ -3270,7 +3270,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="15" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B15" s="2">
         <v>14</v>
       </c>
@@ -3278,7 +3278,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B16" s="2">
         <v>15</v>
       </c>
@@ -3286,7 +3286,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B17" s="2">
         <v>16</v>
       </c>
@@ -3294,7 +3294,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="18" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B18" s="2">
         <v>17</v>
       </c>
@@ -3302,7 +3302,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="19" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B19" s="2">
         <v>18</v>
       </c>
@@ -3310,7 +3310,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="20" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B20" s="2">
         <v>19</v>
       </c>
@@ -3318,7 +3318,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B21" s="2">
         <v>20</v>
       </c>
@@ -3326,7 +3326,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="22" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B22" s="2">
         <v>21</v>
       </c>
@@ -3334,7 +3334,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="23" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B23" s="2">
         <v>22</v>
       </c>
@@ -3342,7 +3342,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="24" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B24" s="2">
         <v>23</v>
       </c>
@@ -3350,7 +3350,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="25" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B25" s="2">
         <v>24</v>
       </c>
@@ -3358,7 +3358,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="26" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B26" s="2">
         <v>25</v>
       </c>
@@ -3366,7 +3366,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="27" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B27" s="2">
         <v>26</v>
       </c>
@@ -3374,7 +3374,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="28" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B28" s="2">
         <v>27</v>
       </c>
@@ -3382,7 +3382,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="29" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B29" s="2">
         <v>28</v>
       </c>
@@ -3390,7 +3390,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="30" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B30" s="2">
         <v>29</v>
       </c>
@@ -3398,7 +3398,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="31" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B31" s="2">
         <v>30</v>
       </c>
@@ -3406,7 +3406,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="32" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B32" s="2">
         <v>31</v>
       </c>
@@ -3414,7 +3414,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="33" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B33" s="2">
         <v>32</v>
       </c>
@@ -3422,7 +3422,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="34" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B34" s="2">
         <v>33</v>
       </c>
@@ -3430,7 +3430,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="35" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B35" s="2">
         <v>34</v>
       </c>
@@ -3438,7 +3438,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="36" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B36" s="2">
         <v>35</v>
       </c>
@@ -3446,7 +3446,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="37" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B37" s="2">
         <v>37</v>
       </c>
@@ -3454,7 +3454,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="38" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B38" s="2">
         <v>38</v>
       </c>
@@ -3462,7 +3462,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="39" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B39" s="2">
         <v>39</v>
       </c>
@@ -3470,7 +3470,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="40" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B40" s="2">
         <v>40</v>
       </c>
@@ -3478,7 +3478,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="41" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B41" s="2">
         <v>41</v>
       </c>
@@ -3486,7 +3486,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="42" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B42" s="2">
         <v>42</v>
       </c>
@@ -3494,7 +3494,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="43" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B43" s="2">
         <v>43</v>
       </c>
@@ -3502,7 +3502,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="44" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B44" s="2">
         <v>44</v>
       </c>
@@ -3510,7 +3510,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="45" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B45" s="2">
         <v>45</v>
       </c>
@@ -3518,7 +3518,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B46" s="2">
         <v>46</v>
       </c>
@@ -3526,7 +3526,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="47" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B47" s="2">
         <v>47</v>
       </c>
@@ -3534,7 +3534,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="48" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B48" s="2">
         <v>48</v>
       </c>
@@ -3542,7 +3542,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="49" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B49" s="2">
         <v>49</v>
       </c>
@@ -3550,7 +3550,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="50" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B50" s="2">
         <v>50</v>
       </c>
@@ -3558,7 +3558,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="51" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B51" s="2">
         <v>51</v>
       </c>
@@ -3566,7 +3566,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="52" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B52" s="2">
         <v>52</v>
       </c>
@@ -3574,7 +3574,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="53" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B53" s="2">
         <v>53</v>
       </c>
@@ -3582,7 +3582,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="54" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B54" s="2">
         <v>54</v>
       </c>
@@ -3590,7 +3590,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="55" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B55" s="2">
         <v>55</v>
       </c>
@@ -3598,7 +3598,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="56" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B56" s="2">
         <v>56</v>
       </c>
@@ -3606,7 +3606,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="57" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B57" s="2">
         <v>57</v>
       </c>
@@ -3614,7 +3614,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="58" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B58" s="2">
         <v>58</v>
       </c>
@@ -3622,7 +3622,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="59" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B59" s="2">
         <v>60</v>
       </c>
@@ -3630,7 +3630,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="60" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B60" s="2">
         <v>61</v>
       </c>
@@ -3638,7 +3638,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="61" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B61" s="2">
         <v>62</v>
       </c>
@@ -3646,7 +3646,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="62" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B62" s="2">
         <v>63</v>
       </c>
@@ -3654,7 +3654,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="63" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B63" s="2">
         <v>64</v>
       </c>
@@ -3662,7 +3662,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="64" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B64" s="2">
         <v>65</v>
       </c>
@@ -3670,7 +3670,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="65" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B65" s="2">
         <v>66</v>
       </c>
@@ -3678,67 +3678,67 @@
         <v>12</v>
       </c>
     </row>
-    <row r="66" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C66" s="8" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="67" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C67" s="5" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="68" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C68" s="5" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="69" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C69" s="5" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="70" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C70" s="8" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="71" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C71" s="8" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="72" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C72" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="73" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C73" s="5" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="74" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C74" s="8" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="75" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C75" s="5" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="76" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C76" s="8" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="77" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C77" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="78" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C78" s="8" t="s">
         <v>93</v>
       </c>
@@ -3748,24 +3748,25 @@
     <sortCondition ref="C87"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B2:L67"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="9.109375" style="1"/>
+    <col min="1" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
       <c r="L2" s="1">
         <f>1971-2024</f>
         <v>-53</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="2">
         <v>1</v>
       </c>
@@ -3773,7 +3774,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="6" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B6" s="2">
         <v>2</v>
       </c>
@@ -3781,7 +3782,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B7" s="2">
         <v>3</v>
       </c>
@@ -3789,7 +3790,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="8" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B8" s="2">
         <v>4</v>
       </c>
@@ -3797,7 +3798,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="9" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="2">
         <v>5</v>
       </c>
@@ -3805,7 +3806,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B10" s="2">
         <v>6</v>
       </c>
@@ -3813,7 +3814,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B11" s="2">
         <v>7</v>
       </c>
@@ -3821,7 +3822,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B12" s="2">
         <v>9</v>
       </c>
@@ -3829,7 +3830,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="13" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B13" s="2">
         <v>10</v>
       </c>
@@ -3837,7 +3838,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B14" s="2">
         <v>12</v>
       </c>
@@ -3845,7 +3846,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="15" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B15" s="2">
         <v>13</v>
       </c>
@@ -3853,7 +3854,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="16" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B16" s="2">
         <v>14</v>
       </c>
@@ -3861,7 +3862,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B17" s="2">
         <v>15</v>
       </c>
@@ -3869,7 +3870,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="18" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B18" s="2">
         <v>16</v>
       </c>
@@ -3877,7 +3878,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="19" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B19" s="2">
         <v>17</v>
       </c>
@@ -3885,7 +3886,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="20" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B20" s="2">
         <v>19</v>
       </c>
@@ -3893,7 +3894,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="21" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B21" s="2">
         <v>20</v>
       </c>
@@ -3901,7 +3902,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="22" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B22" s="2">
         <v>21</v>
       </c>
@@ -3909,7 +3910,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="23" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B23" s="2">
         <v>22</v>
       </c>
@@ -3917,7 +3918,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="24" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B24" s="2">
         <v>23</v>
       </c>
@@ -3925,7 +3926,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="25" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B25" s="2">
         <v>24</v>
       </c>
@@ -3933,7 +3934,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="26" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B26" s="2">
         <v>25</v>
       </c>
@@ -3941,7 +3942,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="27" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B27" s="2">
         <v>27</v>
       </c>
@@ -3949,7 +3950,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="28" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B28" s="2">
         <v>28</v>
       </c>
@@ -3957,102 +3958,102 @@
         <v>122</v>
       </c>
     </row>
-    <row r="29" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C29" s="2" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="30" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C30" s="3" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="31" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C31" s="2" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="32" spans="2:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C32" s="2" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="33" spans="3:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C33" s="3" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="34" spans="3:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="34" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C34" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="3:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="35" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C35" s="2" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="36" spans="3:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="36" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C36" s="2" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="37" spans="3:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="3:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C37" s="2"/>
     </row>
-    <row r="52" spans="5:12" x14ac:dyDescent="0.3">
+    <row r="52" spans="5:12" x14ac:dyDescent="0.25">
       <c r="L52" s="1">
         <v>48120</v>
       </c>
     </row>
-    <row r="53" spans="5:12" x14ac:dyDescent="0.3">
+    <row r="53" spans="5:12" x14ac:dyDescent="0.25">
       <c r="L53" s="1">
         <v>21505</v>
       </c>
     </row>
-    <row r="54" spans="5:12" x14ac:dyDescent="0.3">
+    <row r="54" spans="5:12" x14ac:dyDescent="0.25">
       <c r="L54" s="1">
         <v>19737</v>
       </c>
     </row>
-    <row r="56" spans="5:12" x14ac:dyDescent="0.3">
+    <row r="56" spans="5:12" x14ac:dyDescent="0.25">
       <c r="L56" s="1">
         <f>SUM(L52:L54)</f>
         <v>89362</v>
       </c>
     </row>
-    <row r="59" spans="5:12" x14ac:dyDescent="0.3">
+    <row r="59" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E59" s="1">
         <v>60000</v>
       </c>
     </row>
-    <row r="60" spans="5:12" x14ac:dyDescent="0.3">
+    <row r="60" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E60" s="1">
         <v>6800</v>
       </c>
     </row>
-    <row r="61" spans="5:12" x14ac:dyDescent="0.3">
+    <row r="61" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E61" s="1">
         <v>19000</v>
       </c>
     </row>
-    <row r="62" spans="5:12" x14ac:dyDescent="0.3">
+    <row r="62" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E62" s="1">
         <v>400</v>
       </c>
     </row>
-    <row r="64" spans="5:12" x14ac:dyDescent="0.3">
+    <row r="64" spans="5:12" x14ac:dyDescent="0.25">
       <c r="E64" s="1">
         <f>SUM(E59:E62)</f>
         <v>86200</v>
       </c>
     </row>
-    <row r="65" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="65" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E65" s="1">
         <v>2016</v>
       </c>
     </row>
-    <row r="67" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="67" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E67" s="1">
         <f>SUM(E64:E65)</f>
         <v>88216</v>
@@ -4070,14 +4071,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A4:B87"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="1"/>
-    <col min="2" max="2" width="115.88671875" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.109375" style="1"/>
+    <col min="1" max="1" width="9.140625" style="1"/>
+    <col min="2" max="2" width="115.85546875" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>1</v>
       </c>
@@ -4085,7 +4086,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>2</v>
       </c>
@@ -4093,7 +4094,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>3</v>
       </c>
@@ -4101,7 +4102,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>4</v>
       </c>
@@ -4109,7 +4110,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>5</v>
       </c>
@@ -4117,7 +4118,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>6</v>
       </c>
@@ -4125,7 +4126,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>7</v>
       </c>
@@ -4133,7 +4134,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>8</v>
       </c>
@@ -4141,7 +4142,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>9</v>
       </c>
@@ -4149,7 +4150,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>10</v>
       </c>
@@ -4157,7 +4158,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>11</v>
       </c>
@@ -4165,7 +4166,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>12</v>
       </c>
@@ -4173,7 +4174,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>13</v>
       </c>
@@ -4181,7 +4182,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>14</v>
       </c>
@@ -4189,7 +4190,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>15</v>
       </c>
@@ -4197,7 +4198,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>16</v>
       </c>
@@ -4205,7 +4206,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>17</v>
       </c>
@@ -4213,7 +4214,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>18</v>
       </c>
@@ -4221,7 +4222,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>19</v>
       </c>
@@ -4229,7 +4230,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>20</v>
       </c>
@@ -4237,7 +4238,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>21</v>
       </c>
@@ -4245,7 +4246,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>22</v>
       </c>
@@ -4253,7 +4254,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
         <v>23</v>
       </c>
@@ -4261,7 +4262,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
         <v>24</v>
       </c>
@@ -4269,7 +4270,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
         <v>25</v>
       </c>
@@ -4277,7 +4278,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>26</v>
       </c>
@@ -4285,7 +4286,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
         <v>27</v>
       </c>
@@ -4293,7 +4294,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
         <v>28</v>
       </c>
@@ -4301,7 +4302,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>29</v>
       </c>
@@ -4309,7 +4310,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
         <v>30</v>
       </c>
@@ -4317,7 +4318,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
         <v>31</v>
       </c>
@@ -4325,7 +4326,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="35" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>32</v>
       </c>
@@ -4333,7 +4334,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>33</v>
       </c>
@@ -4341,7 +4342,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
         <v>34</v>
       </c>
@@ -4349,7 +4350,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="38" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
         <v>35</v>
       </c>
@@ -4357,7 +4358,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>36</v>
       </c>
@@ -4365,7 +4366,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>37</v>
       </c>
@@ -4373,7 +4374,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>38</v>
       </c>
@@ -4381,7 +4382,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
         <v>39</v>
       </c>
@@ -4389,7 +4390,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
         <v>40</v>
       </c>
@@ -4397,7 +4398,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="44" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
         <v>41</v>
       </c>
@@ -4405,7 +4406,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="45" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
         <v>42</v>
       </c>
@@ -4413,7 +4414,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="46" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
         <v>43</v>
       </c>
@@ -4421,7 +4422,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="47" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
         <v>44</v>
       </c>
@@ -4429,202 +4430,202 @@
         <v>334</v>
       </c>
     </row>
-    <row r="48" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B48" s="3" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="49" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B49" s="2" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="50" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B50" s="3" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="51" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B51" s="2" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="52" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B52" s="3" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="53" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B53" s="2" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="54" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B54" s="2" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="55" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B55" s="3" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="56" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B56" s="3" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="57" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B57" s="3" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="58" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B58" s="3" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="59" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B59" s="2" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="60" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B60" s="3" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="61" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B61" s="3" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="62" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B62" s="2" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="63" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B63" s="2" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="64" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B64" s="2" t="s">
         <v>269</v>
       </c>
     </row>
-    <row r="65" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B65" s="3" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="66" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B66" s="3" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="67" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B67" s="3" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="68" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B68" s="3" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="69" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B69" s="3" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="70" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B70" s="3" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="71" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B71" s="2" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="72" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B72" s="2" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="73" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B73" s="3" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="74" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B74" s="2" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="75" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B75" s="2" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="76" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B76" s="3" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="77" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B77" s="2" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="78" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B78" s="2" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="79" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B79" s="2" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="80" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B80" s="2" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="81" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B81" s="3" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="82" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B82" s="3" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="83" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B83" s="3" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="84" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B84" s="2" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="85" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B85" s="2" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="86" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B86" s="3" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="87" spans="2:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B87" s="2" t="s">
         <v>433</v>
       </c>
@@ -4638,19 +4639,19 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:L107"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="1"/>
-    <col min="2" max="2" width="71.88671875" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.109375" style="1"/>
+    <col min="1" max="1" width="9.140625" style="1"/>
+    <col min="2" max="2" width="71.85546875" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="L1" s="1" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>1</v>
       </c>
@@ -4661,7 +4662,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>2</v>
       </c>
@@ -4672,7 +4673,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>3</v>
       </c>
@@ -4683,7 +4684,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>4</v>
       </c>
@@ -4694,7 +4695,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>5</v>
       </c>
@@ -4705,7 +4706,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>6</v>
       </c>
@@ -4716,7 +4717,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>7</v>
       </c>
@@ -4727,7 +4728,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>8</v>
       </c>
@@ -4738,7 +4739,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>9</v>
       </c>
@@ -4749,7 +4750,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -4760,7 +4761,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -4771,7 +4772,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -4782,7 +4783,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -4793,7 +4794,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -4804,7 +4805,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -4815,7 +4816,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>17</v>
       </c>
@@ -4826,7 +4827,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -4837,7 +4838,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -4848,7 +4849,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>20</v>
       </c>
@@ -4859,7 +4860,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>21</v>
       </c>
@@ -4870,7 +4871,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -4881,7 +4882,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -4892,7 +4893,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -4903,7 +4904,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -4914,7 +4915,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -4925,7 +4926,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -4936,7 +4937,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -4947,7 +4948,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -4958,7 +4959,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -4969,7 +4970,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -4980,7 +4981,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -4991,7 +4992,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -5002,7 +5003,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -5013,7 +5014,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -5024,7 +5025,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -5035,7 +5036,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -5046,7 +5047,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -5057,7 +5058,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -5068,7 +5069,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -5079,7 +5080,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -5090,7 +5091,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>43</v>
       </c>
@@ -5101,7 +5102,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>44</v>
       </c>
@@ -5112,7 +5113,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>45</v>
       </c>
@@ -5123,7 +5124,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>46</v>
       </c>
@@ -5134,7 +5135,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>47</v>
       </c>
@@ -5145,7 +5146,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>48</v>
       </c>
@@ -5156,7 +5157,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>49</v>
       </c>
@@ -5167,7 +5168,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>50</v>
       </c>
@@ -5178,7 +5179,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>51</v>
       </c>
@@ -5189,7 +5190,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>52</v>
       </c>
@@ -5200,7 +5201,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>53</v>
       </c>
@@ -5211,7 +5212,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>54</v>
       </c>
@@ -5222,7 +5223,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>55</v>
       </c>
@@ -5233,7 +5234,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>56</v>
       </c>
@@ -5244,7 +5245,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>57</v>
       </c>
@@ -5255,7 +5256,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>58</v>
       </c>
@@ -5266,7 +5267,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>59</v>
       </c>
@@ -5277,7 +5278,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="61" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>60</v>
       </c>
@@ -5288,7 +5289,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="62" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>61</v>
       </c>
@@ -5299,7 +5300,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="63" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>62</v>
       </c>
@@ -5310,7 +5311,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>63</v>
       </c>
@@ -5321,7 +5322,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="65" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>64</v>
       </c>
@@ -5332,7 +5333,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="66" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>65</v>
       </c>
@@ -5343,7 +5344,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="67" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>66</v>
       </c>
@@ -5354,7 +5355,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="68" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>67</v>
       </c>
@@ -5365,7 +5366,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="69" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>68</v>
       </c>
@@ -5376,7 +5377,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="70" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>69</v>
       </c>
@@ -5387,7 +5388,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="71" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>70</v>
       </c>
@@ -5398,7 +5399,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="72" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>71</v>
       </c>
@@ -5409,7 +5410,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="73" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>72</v>
       </c>
@@ -5420,7 +5421,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="74" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>73</v>
       </c>
@@ -5431,7 +5432,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="75" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
         <v>74</v>
       </c>
@@ -5442,7 +5443,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="76" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
         <v>75</v>
       </c>
@@ -5453,7 +5454,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="77" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>76</v>
       </c>
@@ -5464,7 +5465,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="78" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
         <v>77</v>
       </c>
@@ -5475,7 +5476,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="79" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
         <v>78</v>
       </c>
@@ -5486,7 +5487,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="80" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
         <v>79</v>
       </c>
@@ -5497,7 +5498,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="81" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
         <v>80</v>
       </c>
@@ -5508,7 +5509,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="82" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
         <v>81</v>
       </c>
@@ -5519,7 +5520,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="83" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
         <v>82</v>
       </c>
@@ -5530,7 +5531,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="84" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
         <v>83</v>
       </c>
@@ -5541,7 +5542,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="85" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
         <v>84</v>
       </c>
@@ -5552,7 +5553,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="86" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
         <v>85</v>
       </c>
@@ -5563,7 +5564,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="87" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
         <v>86</v>
       </c>
@@ -5574,7 +5575,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="88" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
         <v>87</v>
       </c>
@@ -5585,7 +5586,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="89" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
         <v>88</v>
       </c>
@@ -5596,7 +5597,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="90" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
         <v>89</v>
       </c>
@@ -5607,7 +5608,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="91" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
         <v>90</v>
       </c>
@@ -5618,7 +5619,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="92" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
         <v>91</v>
       </c>
@@ -5629,7 +5630,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="93" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
         <v>92</v>
       </c>
@@ -5640,7 +5641,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="94" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
         <v>93</v>
       </c>
@@ -5651,7 +5652,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="95" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
         <v>94</v>
       </c>
@@ -5662,7 +5663,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="96" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
         <v>95</v>
       </c>
@@ -5673,7 +5674,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="97" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
         <v>96</v>
       </c>
@@ -5684,7 +5685,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="98" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
         <v>97</v>
       </c>
@@ -5695,7 +5696,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="99" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
         <v>98</v>
       </c>
@@ -5706,7 +5707,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="100" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
         <v>99</v>
       </c>
@@ -5717,7 +5718,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="101" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
         <v>100</v>
       </c>
@@ -5728,37 +5729,37 @@
         <v>100</v>
       </c>
     </row>
-    <row r="102" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B102" s="2"/>
       <c r="C102" s="1">
         <v>101</v>
       </c>
     </row>
-    <row r="103" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B103" s="2"/>
       <c r="C103" s="1">
         <v>102</v>
       </c>
     </row>
-    <row r="104" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B104" s="2"/>
       <c r="C104" s="1">
         <v>103</v>
       </c>
     </row>
-    <row r="105" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B105" s="2"/>
       <c r="C105" s="1">
         <v>104</v>
       </c>
     </row>
-    <row r="106" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B106" s="2"/>
       <c r="C106" s="1">
         <v>105</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C107" s="1">
         <v>106</v>
       </c>

</xml_diff>